<commit_message>
Stage 8 review fixes: G-011
</commit_message>
<xml_diff>
--- a/output/heldback_firm_G/OsterquillData/Studies/OT-26-S0192/Raw_Observations/Interim/VM14_MN_092426_INTERIM.xlsx
+++ b/output/heldback_firm_G/OsterquillData/Studies/OT-26-S0192/Raw_Observations/Interim/VM14_MN_092426_INTERIM.xlsx
@@ -190,7 +190,7 @@
   <commentList>
     <comment ref="A2" authorId="0" shapeId="0">
       <text>
-        <t>Second reader not yet done on the 3 h +S9 conditions. Hold the mammalian read until that is in.</t>
+        <t>Control acceptance and repeat-condition decisions remain pending. Reconcile exposure records before releasing a final mammalian interpretation.</t>
       </text>
     </comment>
   </commentList>
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>OT-26-S0192 VM14 screen: INTERIM observations, not final</t>
+          <t>Osterquill Toxicology Inc | OT-26-S0192 VM14 screen: INTERIM observations, not final</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Test articles</t>
+          <t>Planned test article cohort</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
@@ -649,7 +649,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>High-concentration conditions excluded for precipitation. Repeats not yet run.</t>
+          <t>Precipitation limited initial high-concentration exposures; condition-specific exclusions and repeat decisions remain to be reconciled with exposure records.</t>
         </is>
       </c>
     </row>
@@ -918,13 +918,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -937,12 +941,9 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Conditions still to be scored are left blank below.</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
+          <t>Pending conditions are tracked at the right; blanks indicate no result entered, not a negative finding.</t>
+        </is>
+      </c>
     </row>
     <row r="3"/>
     <row r="4">
@@ -966,6 +967,27 @@
           <t>RPD (%)</t>
         </is>
       </c>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Pending treatment</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Concentration (µg/mL)</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>MN scoring</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>RPD</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -984,6 +1006,17 @@
       <c r="D5" s="2" t="n">
         <v>100</v>
       </c>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>3 h -S9</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1000,6 +1033,17 @@
       <c r="D6" s="2" t="n">
         <v>95</v>
       </c>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>3 h -S9</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1016,6 +1060,19 @@
       <c r="D7" s="2" t="n">
         <v>82</v>
       </c>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>24 h -S9</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>vehicle</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1032,6 +1089,17 @@
       <c r="D8" s="2" t="n">
         <v>78</v>
       </c>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>24 h -S9</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1050,6 +1118,17 @@
       <c r="D9" s="2" t="n">
         <v>100</v>
       </c>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>24 h -S9</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1066,6 +1145,17 @@
       <c r="D10" s="2" t="n">
         <v>95</v>
       </c>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>24 h -S9</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="n"/>
     </row>
     <row r="11"/>
     <row r="12">

</xml_diff>